<commit_message>
update T column image format: inherit template anchor (54x66px, colOff/rowOff)
</commit_message>
<xml_diff>
--- a/templates/蜡烛-模版.xlsx
+++ b/templates/蜡烛-模版.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="18700"/>
+    <workbookView windowWidth="24620" windowHeight="7720"/>
   </bookViews>
   <sheets>
     <sheet name="下单模板" sheetId="1" r:id="rId1"/>
@@ -1655,13 +1655,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="宋体"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="微软雅黑"/>
+      <name val="宋体"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1672,7 +1672,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1693,19 +1693,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFD8D8D8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD8D8D8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2119,7 +2113,7 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2143,16 +2137,16 @@
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="10" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="8" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -2161,85 +2155,85 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
@@ -2249,7 +2243,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2372,31 +2366,16 @@
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="19" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2417,31 +2396,19 @@
     <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2737,19 +2704,19 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
+      <xdr:colOff>140970</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
+      <xdr:rowOff>71755</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>444500</xdr:colOff>
+      <xdr:colOff>480695</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>500380</xdr:rowOff>
+      <xdr:rowOff>486410</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPr id="2" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -2762,8 +2729,350 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18881725" y="3527425"/>
+          <a:off x="15506065" y="3513455"/>
           <a:ext cx="339725" cy="414655"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>154940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15520035" y="4000500"/>
+          <a:ext cx="311785" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>154940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15520035" y="4000500"/>
+          <a:ext cx="311785" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>154940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15520035" y="4000500"/>
+          <a:ext cx="311785" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>154940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15520035" y="4000500"/>
+          <a:ext cx="311785" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>154940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15520035" y="4000500"/>
+          <a:ext cx="311785" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>154940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15520035" y="4000500"/>
+          <a:ext cx="311785" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>154940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15520035" y="4000500"/>
+          <a:ext cx="311785" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>154940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15520035" y="4000500"/>
+          <a:ext cx="311785" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>154940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="ID_861421884BC9410ABE6122DFE66AA693" descr="wecom-temp-9578-e63d9d2863b1655e589b083bc42b0425"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15520035" y="4000500"/>
+          <a:ext cx="311785" cy="381000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3182,246 +3491,215 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:X5"/>
-  <sheetFormatPr defaultColWidth="8.88461538461539" defaultRowHeight="16.8" outlineLevelRow="4"/>
+  <dimension ref="A1:X4"/>
+  <sheetFormatPr defaultColWidth="8.88461538461539" defaultRowHeight="16.8" outlineLevelRow="3"/>
   <cols>
-    <col min="1" max="1" width="17.4423076923077" style="43" customWidth="1"/>
+    <col min="1" max="1" width="17.4423076923077" customWidth="1"/>
     <col min="2" max="2" width="13.5576923076923" customWidth="1"/>
-    <col min="3" max="3" width="26.2307692307692" style="43" customWidth="1"/>
-    <col min="4" max="4" width="8.88461538461539" style="44"/>
-    <col min="5" max="5" width="36.7692307692308" style="43" customWidth="1"/>
-    <col min="6" max="6" width="11.1538461538462" customWidth="1"/>
-    <col min="7" max="7" width="9.77884615384615" customWidth="1"/>
-    <col min="8" max="8" width="13.3076923076923" customWidth="1"/>
-    <col min="9" max="9" width="30.5384615384615" customWidth="1"/>
+    <col min="3" max="3" width="26.2307692307692" customWidth="1"/>
+    <col min="6" max="7" width="9.77884615384615" customWidth="1"/>
+    <col min="8" max="8" width="12.5576923076923" customWidth="1"/>
     <col min="10" max="10" width="14.2692307692308" customWidth="1"/>
     <col min="11" max="11" width="14.6346153846154" customWidth="1"/>
     <col min="12" max="12" width="14.7788461538462" customWidth="1"/>
-    <col min="15" max="15" width="8.88461538461539" style="44"/>
     <col min="18" max="18" width="15.7788461538462" customWidth="1"/>
     <col min="19" max="19" width="12.7788461538462" customWidth="1"/>
-    <col min="21" max="24" width="15.7788461538462" style="44" customWidth="1"/>
+    <col min="21" max="24" width="15.7788461538462" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="42" customFormat="1" ht="61" customHeight="1" spans="1:24">
-      <c r="A1" s="45" t="s">
+    <row r="1" ht="61" customHeight="1" spans="1:24">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="48"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="48"/>
-      <c r="V1" s="48"/>
-      <c r="W1" s="48"/>
-      <c r="X1" s="49"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="43"/>
+      <c r="U1" s="43"/>
+      <c r="V1" s="43"/>
+      <c r="W1" s="43"/>
+      <c r="X1" s="44"/>
     </row>
-    <row r="2" s="42" customFormat="1" ht="177" customHeight="1" spans="1:24">
-      <c r="A2" s="50" t="s">
+    <row r="2" ht="177" customHeight="1" spans="1:24">
+      <c r="A2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="50" t="s">
+      <c r="B2" s="46"/>
+      <c r="C2" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="52" t="s">
+      <c r="D2" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="50" t="s">
+      <c r="E2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="53"/>
-      <c r="G2" s="50" t="s">
+      <c r="F2" s="48"/>
+      <c r="G2" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="53"/>
-      <c r="I2" s="50" t="s">
+      <c r="H2" s="48"/>
+      <c r="I2" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="53"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="54"/>
-      <c r="O2" s="55" t="s">
+      <c r="J2" s="48"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="P2" s="56"/>
-      <c r="Q2" s="56"/>
-      <c r="R2" s="56"/>
-      <c r="S2" s="50" t="s">
+      <c r="P2" s="51"/>
+      <c r="Q2" s="51"/>
+      <c r="R2" s="51"/>
+      <c r="S2" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="T2" s="57" t="s">
+      <c r="T2" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="U2" s="58"/>
-      <c r="V2" s="58"/>
-      <c r="W2" s="58"/>
-      <c r="X2" s="59"/>
+      <c r="U2" s="52"/>
+      <c r="V2" s="52"/>
+      <c r="W2" s="52"/>
+      <c r="X2" s="49"/>
     </row>
     <row r="3" ht="33" customHeight="1" spans="1:24">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="60" t="s">
+      <c r="C3" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="60" t="s">
+      <c r="D3" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="60" t="s">
+      <c r="E3" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="62" t="s">
+      <c r="F3" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="62" t="s">
+      <c r="G3" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="62" t="s">
+      <c r="H3" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="62" t="s">
+      <c r="I3" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="62" t="s">
+      <c r="J3" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="62" t="s">
+      <c r="K3" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="62" t="s">
+      <c r="L3" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="M3" s="62" t="s">
+      <c r="M3" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="62" t="s">
+      <c r="N3" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="60" t="s">
+      <c r="O3" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="P3" s="62" t="s">
+      <c r="P3" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="Q3" s="62" t="s">
+      <c r="Q3" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="R3" s="62" t="s">
+      <c r="R3" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="S3" s="61" t="s">
+      <c r="S3" s="54" t="s">
         <v>28</v>
       </c>
-      <c r="T3" s="62" t="s">
+      <c r="T3" s="55" t="s">
         <v>29</v>
       </c>
-      <c r="U3" s="60" t="s">
+      <c r="U3" s="53" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="60" t="s">
+      <c r="V3" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="W3" s="60" t="s">
+      <c r="W3" s="53" t="s">
         <v>32</v>
       </c>
-      <c r="X3" s="60" t="s">
+      <c r="X3" s="53" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:24">
-      <c r="A4" s="63"/>
-      <c r="B4" s="64" t="s">
+      <c r="A4" s="56"/>
+      <c r="B4" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="63"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="66" t="s">
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="66" t="s">
+      <c r="G4" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="66" t="s">
+      <c r="H4" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="66" t="s">
+      <c r="I4" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="J4" s="66" t="s">
+      <c r="J4" s="57" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="66">
+      <c r="K4" s="57">
         <v>3406000090</v>
       </c>
-      <c r="L4" s="67"/>
-      <c r="M4" s="66" t="s">
+      <c r="L4" s="58"/>
+      <c r="M4" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="N4" s="66" t="s">
+      <c r="N4" s="57" t="s">
         <v>41</v>
       </c>
-      <c r="O4" s="65"/>
-      <c r="P4" s="66" t="s">
+      <c r="O4" s="56"/>
+      <c r="P4" s="57" t="s">
         <v>42</v>
       </c>
-      <c r="Q4" s="66" t="s">
+      <c r="Q4" s="57" t="s">
         <v>43</v>
       </c>
-      <c r="R4" s="66"/>
-      <c r="S4" s="64"/>
-      <c r="T4" s="66"/>
-      <c r="U4" s="65"/>
-      <c r="V4" s="65"/>
-      <c r="W4" s="65"/>
-      <c r="X4" s="65"/>
-    </row>
-    <row r="5" ht="44" customHeight="1" spans="1:24">
-      <c r="A5" s="63"/>
-      <c r="B5" s="64"/>
-      <c r="C5" s="63"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
-      <c r="H5" s="66"/>
-      <c r="I5" s="66"/>
-      <c r="J5" s="66"/>
-      <c r="K5" s="66"/>
-      <c r="L5" s="67"/>
-      <c r="M5" s="66"/>
-      <c r="N5" s="66"/>
-      <c r="O5" s="65"/>
-      <c r="P5" s="66"/>
-      <c r="Q5" s="66"/>
-      <c r="R5" s="66"/>
-      <c r="S5" s="64"/>
-      <c r="T5" s="66"/>
-      <c r="U5" s="65"/>
-      <c r="V5" s="65"/>
-      <c r="W5" s="65"/>
-      <c r="X5" s="65"/>
+      <c r="R4" s="57"/>
+      <c r="S4" s="56"/>
+      <c r="T4" s="57"/>
+      <c r="U4" s="56"/>
+      <c r="V4" s="56"/>
+      <c r="W4" s="56"/>
+      <c r="X4" s="56"/>
     </row>
   </sheetData>
   <protectedRanges>

</xml_diff>